<commit_message>
refined generate artifacts logic for big log files
</commit_message>
<xml_diff>
--- a/UAT_Excel_Reports/Bbu Alerts_UAT.xlsx
+++ b/UAT_Excel_Reports/Bbu Alerts_UAT.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F148"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -496,26 +496,39 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>--- INITIAL NAVIGATION TO DASHBOARD ---</t>
-        </is>
-      </c>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>C.1</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Navigate to the 'Executive Dashboard' in the demand planning application by entering the specified URL in the browser.</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>`page.goto("https://stage.bbu.esp.antuit.ai/dp/demand-planning/executive-dashboard?workbookId=4&amp;tabIndex=1")`</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>C.1</t>
+          <t>D.1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Navigate to the 'Executive Dashboard' in the demand planning application by entering the specified URL in the browser.</t>
+          <t>Click on the 'Filter' button to open the filter options in the dashboard.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>`page.goto("https://stage.bbu.esp.antuit.ai/dp/demand-planning/executive-dashboard?workbookId=4&amp;tabIndex=1")`</t>
+          <t>`page.get_by_text("Filter").click()`</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -523,26 +536,39 @@
       <c r="F4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>--- FILTER INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>D.2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>From the filter dropdown, select the 'Alerts' option to filter by alerts.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("#alerts-filterId").get_by_text("Alerts").click()`</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>D.1</t>
+          <t>D.3</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter' button to open the filter options in the dashboard.</t>
+          <t>Click on the dropdown caret to expand the filter options.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Filter").click()`</t>
+          <t>`page.locator(".dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -552,17 +578,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>D.2</t>
+          <t>D.4</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>From the filter dropdown, select the 'Alerts' option to filter by alerts.</t>
+          <t>From the expanded dropdown, select the 'Over Bias' filter option.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#alerts-filterId").get_by_text("Alerts").click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Over Bias$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -572,12 +598,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>D.3</t>
+          <t>D.5</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret to expand the filter options.</t>
+          <t>Click on the dropdown caret again to expand the filter options.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -592,17 +618,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>D.4</t>
+          <t>D.6</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Over Bias' filter option.</t>
+          <t>From the expanded dropdown, select the 'Under Bias' filter option.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Over Bias$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Under Bias$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -612,7 +638,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>D.5</t>
+          <t>D.7</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -632,17 +658,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>D.6</t>
+          <t>D.8</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Under Bias' filter option.</t>
+          <t>From the expanded dropdown, select the 'MAPE' filter option.</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Under Bias$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^MAPE$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
@@ -652,7 +678,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>D.7</t>
+          <t>D.9</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -672,17 +698,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>D.8</t>
+          <t>D.10</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'MAPE' filter option.</t>
+          <t>From the expanded dropdown, select the 'Stability' filter option.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^MAPE$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Stability$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -692,7 +718,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>D.9</t>
+          <t>D.11</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -712,17 +738,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>D.10</t>
+          <t>D.12</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Stability' filter option.</t>
+          <t>From the expanded dropdown, select the 'FVA' filter option.</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Stability$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^FVA$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr"/>
@@ -732,17 +758,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>D.11</t>
+          <t>E.1</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to expand the filter options.</t>
+          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".dropdown-caret").first.click()`</t>
+          <t>`page.get_by_role("button", name="columns").click()`</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr"/>
@@ -752,17 +778,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>D.12</t>
+          <t>E.2</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'FVA' filter option.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^FVA$")).nth(1).click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr"/>
@@ -770,26 +796,39 @@
       <c r="F17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>--- COLUMN VISIBILITY CONFIGURATION ---</t>
-        </is>
-      </c>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>E.3</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Uncheck the '6W-Actuals Column' checkbox to hide this specific column.</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("treeitem", name="6W-Actuals Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>E.1</t>
+          <t>E.4</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
+          <t>Uncheck the 'User Bias Column' checkbox to hide this specific column.</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").click()`</t>
+          <t>`page.get_by_role("treeitem", name="User Bias Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
@@ -799,17 +838,17 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>E.2</t>
+          <t>F.1</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>Click on the 'Adjustments' button to open the preferences menu.</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr"/>
@@ -819,17 +858,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>E.3</t>
+          <t>F.2</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the '6W-Actuals Column' checkbox to hide this specific column.</t>
+          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="6W-Actuals Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr"/>
@@ -839,17 +878,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>E.4</t>
+          <t>F.3</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the 'User Bias Column' checkbox to hide this specific column.</t>
+          <t>Click on the 'Download' button to export the saved preferences.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="User Bias Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator(".icon-color-toolbar-active.zeb-download-underline").click()`</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
@@ -857,26 +896,39 @@
       <c r="F22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>--- PREFERENCES AND DOWNLOAD HANDLING ---</t>
-        </is>
-      </c>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>G.1</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Click on the 'Adjustments' button again to reopen the preferences menu.</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>F.1</t>
+          <t>G.2</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Adjustments' button to open the preferences menu.</t>
+          <t>Click on 'Reset Preference' to revert to the default column visibility settings.</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr"/>
@@ -886,17 +938,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>F.2</t>
+          <t>G.3</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
+          <t>Click on the filter icon to open the filter menu for the first column.</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
@@ -906,17 +958,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>F.3</t>
+          <t>G.4</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Download' button to export the saved preferences.</t>
+          <t>Enter 'WINCO' into the filter text box to filter the data by this value.</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".icon-color-toolbar-active.zeb-download-underline").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Value").fill("WINCO")`</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr"/>
@@ -924,26 +976,39 @@
       <c r="F26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>--- FILTER AND STATUS DROPDOWN INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>G.5</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Click on the 'Apply' button to apply the filter and update the data view.</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("button", name="Apply").click()`</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>G.1</t>
+          <t>G.6</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Adjustments' button again to reopen the preferences menu.</t>
+          <t>Click on the filter icon again to reopen the filter menu for the first column.</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
+          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr"/>
@@ -953,17 +1018,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>G.2</t>
+          <t>G.7</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Reset Preference' to revert to the default column visibility settings.</t>
+          <t>Click on the 'Reset' button to clear the applied filter and restore the default data view.</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.get_by_role("button", name="Reset").click()`</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
@@ -973,17 +1038,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>G.3</t>
+          <t>G.8</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon to open the filter menu for the first column.</t>
+          <t>Click on the dropdown caret to open the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
@@ -993,17 +1058,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>G.4</t>
+          <t>G.9</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Enter 'WINCO' into the filter text box to filter the data by this value.</t>
+          <t>Select the 'In progress' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Value").fill("WINCO")`</t>
+          <t>`page.get_by_text("In progress").click()`</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
@@ -1013,17 +1078,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>G.5</t>
+          <t>G.10</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Apply' button to apply the filter and update the data view.</t>
+          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="Apply").click()`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr"/>
@@ -1033,17 +1098,17 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>G.6</t>
+          <t>G.11</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon again to reopen the filter menu for the first column.</t>
+          <t>Select the 'Completed' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
+          <t>`page.get_by_text("Completed").click()`</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr"/>
@@ -1053,17 +1118,17 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>G.7</t>
+          <t>G.12</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset' button to clear the applied filter and restore the default data view.</t>
+          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="Reset").click()`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr"/>
@@ -1073,17 +1138,17 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>G.8</t>
+          <t>G.13</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret to open the dropdown menu for selecting a status.</t>
+          <t>Select the 'Not started' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.get_by_text("Not started").click()`</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr"/>
@@ -1093,17 +1158,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>G.9</t>
+          <t>H.1</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Select the 'In progress' option from the dropdown menu.</t>
+          <t>Double-click on 'WALMART STORES HQ' in the treegrid to expand its details.</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("In progress").click()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").dblclick()`</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr"/>
@@ -1113,17 +1178,17 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>G.10</t>
+          <t>H.2</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
+          <t>Double-click on the first occurrence of the text 'WALMART' to navigate further.</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.locator("span").filter(has_text="WALMART").first.dblclick()`</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
@@ -1133,17 +1198,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>G.11</t>
+          <t>H.3</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Completed' option from the dropdown menu.</t>
+          <t>Double-click on 'WALMART 0906 SC B-0006805-01-' in the treegrid to expand its details.</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Completed").click()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART 0906 SC B-0006805-01-").dblclick()`</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr"/>
@@ -1153,17 +1218,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>G.12</t>
+          <t>H.4</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
+          <t>Right-click on 'WALMART 0906 SC B-0006805-01-' to open the context menu.</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.get_by_text("WALMART 0906 SC B-0006805-01-").click(button="right")`</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr"/>
@@ -1173,17 +1238,17 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>G.13</t>
+          <t>H.5</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Not started' option from the dropdown menu.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Not started").click()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr"/>
@@ -1191,26 +1256,39 @@
       <c r="F40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>--- TREEGRID INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>H.6</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Right-click on the highlighted row in the treegrid to open the context menu.</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".ag-row-even.ag-row-focus.ag-row-not-inline-editing.ag-row.ag-row-level-0.ag-row-position-absolute.ag-row-first.ag-row-hover &gt; .ag-cell-value &gt; .ag-cell-wrapper").click(button="right")`</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>H.1</t>
+          <t>H.7</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Double-click on 'WALMART STORES HQ' in the treegrid to expand its details.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").dblclick()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr"/>
@@ -1220,17 +1298,17 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>H.2</t>
+          <t>H.8</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the first occurrence of the text 'WALMART' to navigate further.</t>
+          <t>Right-click on 'WALMART STORES HQ' in the treegrid to open the context menu.</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("span").filter(has_text="WALMART").first.dblclick()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").click(button="right")`</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr"/>
@@ -1240,17 +1318,17 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>H.3</t>
+          <t>H.9</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Double-click on 'WALMART 0906 SC B-0006805-01-' in the treegrid to expand its details.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART 0906 SC B-0006805-01-").dblclick()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr"/>
@@ -1260,17 +1338,17 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>H.4</t>
+          <t>I.1</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Right-click on 'WALMART 0906 SC B-0006805-01-' to open the context menu.</t>
+          <t>Click on the column header labeled '6W-Actuals' to sort or interact with the column.</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("WALMART 0906 SC B-0006805-01-").click(button="right")`</t>
+          <t>`page.get_by_role("columnheader", name="6W-Actuals").click()`</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr"/>
@@ -1280,17 +1358,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>H.5</t>
+          <t>I.2</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Click on the page number '2' in the pagination control to navigate to the second page of the grid.</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.locator("a").filter(has_text="2").click()`</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr"/>
@@ -1300,17 +1378,17 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>H.6</t>
+          <t>I.3</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Right-click on the highlighted row in the treegrid to open the context menu.</t>
+          <t>Click on the 'First Page' button in the pagination control to navigate to the first page of the grid.</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-row-even.ag-row-focus.ag-row-not-inline-editing.ag-row.ag-row-level-0.ag-row-position-absolute.ag-row-first.ag-row-hover &gt; .ag-cell-value &gt; .ag-cell-wrapper").click(button="right")`</t>
+          <t>`page.locator(".zeb-nav-to-first").click()`</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr"/>
@@ -1320,17 +1398,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>H.7</t>
+          <t>I.4</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Select the row containing 'WALMART STORES HQ' by checking the checkbox in the grid cell.</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.get_by_role("gridcell", name="Press Space to toggle row selection (unchecked)   WALMART STORES HQ").get_by_label("Press Space to toggle row").check()`</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr"/>
@@ -1340,17 +1418,17 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>H.8</t>
+          <t>I.5</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Right-click on 'WALMART STORES HQ' in the treegrid to open the context menu.</t>
+          <t>Uncheck the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").click(button="right")`</t>
+          <t>`page.locator(".checkbox-primary-color").first.uncheck()`</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr"/>
@@ -1360,17 +1438,17 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>H.9</t>
+          <t>I.6</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Check the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
@@ -1378,26 +1456,39 @@
       <c r="F50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>--- PAGINATION AND GRID INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>I.7</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Uncheck the first checkbox in the grid using the '.d-flex.align-items-center.checkbox-primary-color' locator.</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".d-flex.align-items-center.checkbox-primary-color").first.uncheck()`</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="4" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>I.1</t>
+          <t>I.8</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Click on the column header labeled '6W-Actuals' to sort or interact with the column.</t>
+          <t>Uncheck the first checkbox in the grid using a more specific locator targeting a nested structure within the grid.</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("columnheader", name="6W-Actuals").click()`</t>
+          <t>`page.locator(".ag-row-odd &gt; .ag-cell-value &gt; .ag-cell-wrapper &gt; .ag-group-value &gt; aeap-group-cell-renderer &gt; .d-flex.align-items-center.w-fit-content &gt; .d-flex").first.uncheck()`</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr"/>
@@ -1407,17 +1498,17 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>I.2</t>
+          <t>J.1</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Click on the page number '2' in the pagination control to navigate to the second page of the grid.</t>
+          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("a").filter(has_text="2").click()`</t>
+          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr"/>
@@ -1427,17 +1518,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>I.3</t>
+          <t>J.2</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'First Page' button in the pagination control to navigate to the first page of the grid.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".zeb-nav-to-first").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr"/>
@@ -1447,17 +1538,17 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>I.4</t>
+          <t>J.3</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Select the row containing 'WALMART STORES HQ' by checking the checkbox in the grid cell.</t>
+          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell", name="Press Space to toggle row selection (unchecked)   WALMART STORES HQ").get_by_label("Press Space to toggle row").check()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr"/>
@@ -1467,17 +1558,17 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>I.5</t>
+          <t>J.4</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
+          <t>Fill the 'Filter Columns Input' textbox with the text 'User Bias' to filter columns by this keyword.</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.uncheck()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("User Bias")`</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr"/>
@@ -1487,17 +1578,17 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>I.6</t>
+          <t>J.5</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Check the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
+          <t>Uncheck the checkbox corresponding to the 'User Bias' column to hide it.</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
+          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr"/>
@@ -1507,17 +1598,17 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>I.7</t>
+          <t>J.6</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the first checkbox in the grid using the '.d-flex.align-items-center.checkbox-primary-color' locator.</t>
+          <t>Click on the 'Filter Columns Input' textbox again to focus on it.</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".d-flex.align-items-center.checkbox-primary-color").first.uncheck()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr"/>
@@ -1527,17 +1618,17 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>I.8</t>
+          <t>J.7</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the first checkbox in the grid using a more specific locator targeting a nested structure within the grid.</t>
+          <t>Select all text in the 'Filter Columns Input' textbox using the 'ControlOrMeta+a' keyboard shortcut.</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-row-odd &gt; .ag-cell-value &gt; .ag-cell-wrapper &gt; .ag-group-value &gt; aeap-group-cell-renderer &gt; .d-flex.align-items-center.w-fit-content &gt; .d-flex").first.uncheck()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").press("ControlOrMeta+a")`</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr"/>
@@ -1545,26 +1636,39 @@
       <c r="F59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>--- ADVANCED COLUMN VISIBILITY CONFIGURATION ---</t>
-        </is>
-      </c>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>J.8</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Clear the 'Filter Columns Input' textbox by filling it with an empty string.</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("")`</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr"/>
+      <c r="E60" s="4" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>J.1</t>
+          <t>J.9</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox again to ensure all columns are visible.</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr"/>
@@ -1574,17 +1678,17 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>J.2</t>
+          <t>J.10</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>Click on the 'Columns' button to close the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr"/>
@@ -1594,17 +1698,17 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>J.3</t>
+          <t>K.1</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
+          <t>Click on the 'Preference' dropdown menu to open the preference options.</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr"/>
@@ -1614,17 +1718,17 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>J.4</t>
+          <t>K.2</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Fill the 'Filter Columns Input' textbox with the text 'User Bias' to filter columns by this keyword.</t>
+          <t>Click on the 'Save Preference' option to save the current grid settings.</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("User Bias")`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr"/>
@@ -1634,17 +1738,17 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>J.5</t>
+          <t>K.3</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the checkbox corresponding to the 'User Bias' column to hide it.</t>
+          <t>Click on the 'Export' button to export the grid data, triggering a file download.</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div:nth-child(2) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr"/>
@@ -1654,17 +1758,17 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>J.6</t>
+          <t>L.1</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox again to focus on it.</t>
+          <t>Click on the 'Preference' dropdown menu again to reopen the preference options.</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr"/>
@@ -1674,17 +1778,17 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>J.7</t>
+          <t>L.2</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Select all text in the 'Filter Columns Input' textbox using the 'ControlOrMeta+a' keyboard shortcut.</t>
+          <t>Click on the 'Reset Preference' option to revert the grid settings to their default state.</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").press("ControlOrMeta+a")`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr"/>
@@ -1694,17 +1798,17 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>J.8</t>
+          <t>L.3</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Clear the 'Filter Columns Input' textbox by filling it with an empty string.</t>
+          <t>Click on the filter icon in the column header to open the filter options for the selected column.</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("")`</t>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr"/>
@@ -1714,17 +1818,17 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>J.9</t>
+          <t>L.4</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox again to ensure all columns are visible.</t>
+          <t>Enter the filter value '761' into the filter input field to apply a filter to the column.</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_role("spinbutton", name="Filter Value").fill("761")`</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr"/>
@@ -1734,17 +1838,17 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>J.10</t>
+          <t>L.5</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to close the column visibility configuration panel.</t>
+          <t>Click on the 'Apply' button in the column filter menu to apply the filter and update the grid data.</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr"/>
@@ -1752,26 +1856,39 @@
       <c r="F70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>--- PREFERENCE AND EXPORT HANDLING ---</t>
-        </is>
-      </c>
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>L.6</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Click on the filter icon again to reopen the column filter menu after applying the filter.</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="4" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>K.1</t>
+          <t>L.7</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' dropdown menu to open the preference options.</t>
+          <t>Click on the 'Reset' button in the column filter menu to clear the applied filter and restore the grid data to its original state.</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr"/>
@@ -1781,17 +1898,17 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>K.2</t>
+          <t>M.1</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Save Preference' option to save the current grid settings.</t>
+          <t>Check the first checkbox with the primary color styling to select the corresponding row.</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr"/>
@@ -1801,17 +1918,17 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>K.3</t>
+          <t>M.2</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Export' button to export the grid data, triggering a file download.</t>
+          <t>Double-click on the row containing the text 'ENTENMANNS' to drill down into its details.</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(2) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`page.locator("span").filter(has_text="ENTENMANNS").first.dblclick()`</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr"/>
@@ -1819,26 +1936,39 @@
       <c r="F74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>--- COLUMN FILTERING AND RESET ---</t>
-        </is>
-      </c>
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>M.3</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Double-click on the row containing the text 'EN BITES' to further drill down into its details.</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("span").filter(has_text="EN BITES").first.dblclick()`</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="4" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>L.1</t>
+          <t>M.4</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' dropdown menu again to reopen the preference options.</t>
+          <t>Double-click on the row containing the text 'EN LITTLE BITES CP' to navigate deeper into its details.</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_text("EN LITTLE BITES CP").first.dblclick()`</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr"/>
@@ -1848,17 +1978,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>L.2</t>
+          <t>M.5</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset Preference' option to revert the grid settings to their default state.</t>
+          <t>Right-click on the row containing the text 'EN LB CHOCCH MFN 10P-' to open the context menu for additional actions.</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.get_by_text("EN LB CHOCCH MFN 10P-").first.click(button="right")`</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr"/>
@@ -1868,17 +1998,17 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>L.3</t>
+          <t>M.6</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon in the column header to open the filter options for the selected column.</t>
+          <t>Click on the 'Drill up' option in the context menu to navigate back to the previous level.</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr"/>
@@ -1888,17 +2018,17 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>L.4</t>
+          <t>M.7</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Enter the filter value '761' into the filter input field to apply a filter to the column.</t>
+          <t>Right-click on the first grid cell with an empty text value to open the context menu.</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("spinbutton", name="Filter Value").fill("761")`</t>
+          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click(button="right")`</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr"/>
@@ -1908,17 +2038,17 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>L.5</t>
+          <t>M.8</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Apply' button in the column filter menu to apply the filter and update the grid data.</t>
+          <t>Click on the first grid cell with an empty text value to select it.</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
+          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click()`</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr"/>
@@ -1928,17 +2058,17 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>L.6</t>
+          <t>N.1</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon again to reopen the column filter menu after applying the filter.</t>
+          <t>Click on the link within the 'Products' card to navigate to the detailed view of the products.</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
+          <t>`page.locator("esp-card-component").filter(has_text="Products10 rows out of 11").locator("a").click()`</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr"/>
@@ -1948,17 +2078,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>L.7</t>
+          <t>N.2</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset' button in the column filter menu to clear the applied filter and restore the grid data to its original state.</t>
+          <t>Click on the 'First Page' button in the pagination controls to navigate to the first page of the product list.</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first &gt; .zeb-nav-to-first").click()`</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr"/>
@@ -1966,26 +2096,39 @@
       <c r="F82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>--- ROW AND DRILL-DOWN INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>N.3</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Click on the 'Apply' button to apply the selected filters or changes.</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("button", name="Apply").click()`</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr"/>
+      <c r="E83" s="4" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>M.1</t>
+          <t>N.4</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Check the first checkbox with the primary color styling to select the corresponding row.</t>
+          <t>Click on the 'Filter' section to expand or interact with the filter options.</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Filter$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr"/>
@@ -1995,17 +2138,17 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>M.2</t>
+          <t>N.5</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the row containing the text 'ENTENMANNS' to drill down into its details.</t>
+          <t>Click on the dropdown caret in the 'Time' filter to open the dropdown menu.</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("span").filter(has_text="ENTENMANNS").first.dblclick()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr"/>
@@ -2015,17 +2158,17 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>M.3</t>
+          <t>N.6</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the row containing the text 'EN BITES' to further drill down into its details.</t>
+          <t>Select the 'Latest 5 Next 4' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("span").filter(has_text="EN BITES").first.dblclick()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 4$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr"/>
@@ -2035,17 +2178,17 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>M.4</t>
+          <t>N.7</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the row containing the text 'EN LITTLE BITES CP' to navigate deeper into its details.</t>
+          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for a new selection.</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("EN LITTLE BITES CP").first.dblclick()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr"/>
@@ -2055,17 +2198,17 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>M.5</t>
+          <t>N.8</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Right-click on the row containing the text 'EN LB CHOCCH MFN 10P-' to open the context menu for additional actions.</t>
+          <t>Select the 'Latest 5 Next 12' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("EN LB CHOCCH MFN 10P-").first.click(button="right")`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 12$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr"/>
@@ -2075,17 +2218,17 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>M.6</t>
+          <t>N.9</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Drill up' option in the context menu to navigate back to the previous level.</t>
+          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for another selection.</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr"/>
@@ -2095,17 +2238,17 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>M.7</t>
+          <t>N.10</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Right-click on the first grid cell with an empty text value to open the context menu.</t>
+          <t>Select the 'Latest 13 Next 4' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click(button="right")`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 13 Next 4$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr"/>
@@ -2115,17 +2258,17 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>M.8</t>
+          <t>O.1</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Click on the first grid cell with an empty text value to select it.</t>
+          <t>Click on the 'Weekly Summary Customer:' card button to expand or interact with the card.</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click()`</t>
+          <t>`page.locator("esp-card-component").filter(has_text="Weekly Summary Customer:").get_by_role("button").click()`</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr"/>
@@ -2133,26 +2276,39 @@
       <c r="F91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>--- PRODUCT NAVIGATION AND TIME FILTER ---</t>
-        </is>
-      </c>
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>O.2</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Uncheck the visibility toggle for the column labeled '-11-02 (45) Column'.</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("treeitem", name="-11-02 (45) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="4" t="inlineStr"/>
+      <c r="F92" s="4" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>N.1</t>
+          <t>O.3</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Click on the link within the 'Products' card to navigate to the detailed view of the products.</t>
+          <t>Uncheck the visibility toggle for the column labeled '-11-09 (46) Column'.</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Products10 rows out of 11").locator("a").click()`</t>
+          <t>`page.get_by_role("treeitem", name="-11-09 (46) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr"/>
@@ -2162,17 +2318,17 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>N.2</t>
+          <t>O.4</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'First Page' button in the pagination controls to navigate to the first page of the product list.</t>
+          <t>Uncheck the visibility toggle for the column labeled '-11-16 (47) Column'.</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first &gt; .zeb-nav-to-first").click()`</t>
+          <t>`page.get_by_role("treeitem", name="-11-16 (47) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr"/>
@@ -2182,17 +2338,17 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>N.3</t>
+          <t>O.5</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Apply' button to apply the selected filters or changes.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="Apply").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr"/>
@@ -2202,17 +2358,17 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>N.4</t>
+          <t>O.6</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter' section to expand or interact with the filter options.</t>
+          <t>Click on the preference dropdown icon to open the preference options.</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Filter$")).nth(1).click()`</t>
+          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr"/>
@@ -2222,17 +2378,17 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>N.5</t>
+          <t>O.7</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter to open the dropdown menu.</t>
+          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr"/>
@@ -2242,17 +2398,17 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>N.6</t>
+          <t>O.8</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 5 Next 4' option from the 'Time' filter dropdown.</t>
+          <t>Click on the preference dropdown icon again to reopen the preference options.</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 4$")).nth(1).click()`</t>
+          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr"/>
@@ -2262,17 +2418,17 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>N.7</t>
+          <t>O.9</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for a new selection.</t>
+          <t>Click on 'Reset Preference' to reset the column visibility settings to their default state.</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr"/>
@@ -2282,17 +2438,17 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>N.8</t>
+          <t>P.1</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 5 Next 12' option from the 'Time' filter dropdown.</t>
+          <t>Click on the export icon to initiate the download process.</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 12$")).nth(1).click()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr"/>
@@ -2302,17 +2458,17 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>N.9</t>
+          <t>P.2</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for another selection.</t>
+          <t>Click on the first element with the class 'align-middle' to interact with it.</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.locator(".align-middle").first.click()`</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr"/>
@@ -2322,17 +2478,17 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>N.10</t>
+          <t>P.3</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 13 Next 4' option from the 'Time' filter dropdown.</t>
+          <t>Click on the second occurrence of the text 'Event' to navigate or interact with the Event section.</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 13 Next 4$")).nth(1).click()`</t>
+          <t>`page.get_by_text("Event").nth(1).click()`</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr"/>
@@ -2340,26 +2496,39 @@
       <c r="F102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>--- WEEKLY SUMMARY AND COLUMN VISIBILITY ---</t>
-        </is>
-      </c>
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>P.4</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Click on the button within the 'Event Details columns (0)' card to open column visibility options.</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("esp-card-component").filter(has_text="Event Details columns (0)").get_by_role("button").click()`</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr"/>
+      <c r="E103" s="4" t="inlineStr"/>
+      <c r="F103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>O.1</t>
+          <t>P.5</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Weekly Summary Customer:' card button to expand or interact with the card.</t>
+          <t>Uncheck the visibility toggle for the 'Event Column' to hide it.</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Weekly Summary Customer:").get_by_role("button").click()`</t>
+          <t>`page.get_by_role("treeitem", name="Event Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr"/>
@@ -2369,17 +2538,17 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>O.2</t>
+          <t>P.6</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-02 (45) Column'.</t>
+          <t>Uncheck the visibility toggle for the 'UPC 12 Column' to hide it.</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="-11-02 (45) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="UPC 12 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr"/>
@@ -2389,17 +2558,17 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>O.3</t>
+          <t>P.7</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-09 (46) Column'.</t>
+          <t>Uncheck the visibility toggle for the 'Customer Level 2 Column' to hide it.</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="-11-09 (46) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="Customer Level 2 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr"/>
@@ -2409,17 +2578,17 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>O.4</t>
+          <t>P.8</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-16 (47) Column'.</t>
+          <t>Uncheck the visibility toggle for the 'Start Date Column' to hide it.</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="-11-16 (47) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="Start Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr"/>
@@ -2429,17 +2598,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>O.5</t>
+          <t>P.9</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>Uncheck the visibility toggle for the 'End Date Column' to hide it.</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_role("treeitem", name="End Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr"/>
@@ -2449,17 +2618,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>O.6</t>
+          <t>P.10</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Click on the preference dropdown icon to open the preference options.</t>
+          <t>Uncheck the visibility toggle for the 'Max Promo Price Column' to hide it.</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_role("treeitem", name="Max Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr"/>
@@ -2469,17 +2638,17 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>O.7</t>
+          <t>P.11</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
+          <t>Uncheck the visibility toggle for the 'Min Promo Price Column' to hide it.</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.get_by_role("treeitem", name="Min Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr"/>
@@ -2489,17 +2658,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>O.8</t>
+          <t>P.12</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Click on the preference dropdown icon again to reopen the preference options.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible again.</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr"/>
@@ -2509,17 +2678,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>O.9</t>
+          <t>P.13</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Reset Preference' to reset the column visibility settings to their default state.</t>
+          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr"/>
@@ -2527,26 +2696,39 @@
       <c r="F112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>--- EXPORT AND PAGINATION INTERACTIONS ---</t>
-        </is>
-      </c>
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>P.14</t>
+        </is>
+      </c>
+      <c r="B113" s="4" t="inlineStr">
+        <is>
+          <t>Fill the 'Filter Columns Input' textbox with the text 'UPC' to filter columns by this keyword.</t>
+        </is>
+      </c>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("UPC")`</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr"/>
+      <c r="E113" s="4" t="inlineStr"/>
+      <c r="F113" s="4" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>P.1</t>
+          <t>P.15</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Click on the export icon to initiate the download process.</t>
+          <t>Uncheck the visibility toggle for the filtered column matching 'UPC' to hide it.</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr"/>
@@ -2556,17 +2738,17 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>P.2</t>
+          <t>P.16</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Click on the first element with the class 'align-middle' to interact with it.</t>
+          <t>Click on the 'Preference' icon to open the dropdown menu for saving preferences.</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".align-middle").first.click()`</t>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div:nth-child(2) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr"/>
@@ -2576,17 +2758,17 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>P.3</t>
+          <t>P.17</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Click on the second occurrence of the text 'Event' to navigate or interact with the Event section.</t>
+          <t>Click on 'Save Preference' to save the current grid settings or preferences.</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Event").nth(1).click()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr"/>
@@ -2596,17 +2778,17 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>P.4</t>
+          <t>P.18</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Click on the button within the 'Event Details columns (0)' card to open column visibility options.</t>
+          <t>Click on the 'Export' icon to initiate the export process and trigger the file download.</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Event Details columns (0)").get_by_role("button").click()`</t>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr"/>
@@ -2616,17 +2798,17 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>P.5</t>
+          <t>P.19</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Event Column' to hide it.</t>
+          <t>Click on the second page link in the pagination to navigate to the second page of the grid.</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Event Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("a").nth(2).click()`</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr"/>
@@ -2636,17 +2818,17 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>P.6</t>
+          <t>P.20</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'UPC 12 Column' to hide it.</t>
+          <t>Click on the page link labeled '3' to navigate to the third page of the grid.</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="UPC 12 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("a").filter(has_text="3").click()`</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr"/>
@@ -2656,17 +2838,17 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>P.7</t>
+          <t>P.21</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Customer Level 2 Column' to hide it.</t>
+          <t>Click on the 'First Page' button in the pagination controls to navigate back to the first page of the grid.</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Customer Level 2 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .card-content &gt; esp-row-dimentional-grid &gt; div &gt; #paginationId &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first").click()`</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr"/>
@@ -2676,17 +2858,17 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>P.8</t>
+          <t>Q.1</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Start Date Column' to hide it.</t>
+          <t>Click on the dropdown labeled 'View 10 row(s)' to open the row display options.</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Start Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_text("View 10 row(s)").nth(2).click()`</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr"/>
@@ -2696,17 +2878,17 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>P.9</t>
+          <t>Q.2</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'End Date Column' to hide it.</t>
+          <t>Select the option 'View 20 row(s)' from the dropdown to change the number of rows displayed.</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="End Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^View 20 row\(s\)$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr"/>
@@ -2716,17 +2898,17 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>P.10</t>
+          <t>Q.3</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Max Promo Price Column' to hide it.</t>
+          <t>Click on the column header icon to open the filter options for the column.</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Max Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr"/>
@@ -2736,17 +2918,17 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>P.11</t>
+          <t>Q.4</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Min Promo Price Column' to hide it.</t>
+          <t>Fill the filter textbox with the value 'Promotion' to filter the column based on this value.</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Min Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Value").fill("Promotion")`</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr"/>
@@ -2756,17 +2938,17 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>P.12</t>
+          <t>Q.5</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible again.</t>
+          <t>Click the 'Apply' button to apply the column filter.</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr"/>
@@ -2776,17 +2958,17 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>P.13</t>
+          <t>Q.6</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
+          <t>Click on the filtered column header to interact with the column filter settings.</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-cell-filtered &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container").click()`</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr"/>
@@ -2796,17 +2978,17 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>P.14</t>
+          <t>Q.7</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Fill the 'Filter Columns Input' textbox with the text 'UPC' to filter columns by this keyword.</t>
+          <t>Click on the filter icon to open the active filter options for the column.</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("UPC")`</t>
+          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr"/>
@@ -2816,17 +2998,17 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>P.15</t>
+          <t>Q.8</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the filtered column matching 'UPC' to hide it.</t>
+          <t>Click the 'Reset' button to clear the applied column filter.</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr"/>
@@ -2836,17 +3018,17 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>P.16</t>
+          <t>R.1</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' icon to open the dropdown menu for saving preferences.</t>
+          <t>Double-click on the grid cell with the name 'Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/' to interact with or edit the cell.</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div:nth-child(2) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_role("gridcell", name="Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/").dblclick()`</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr"/>
@@ -2856,17 +3038,17 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>P.17</t>
+          <t>R.2</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current grid settings or preferences.</t>
+          <t>Close the current page after completing the interaction.</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.close()`</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr"/>
@@ -2876,17 +3058,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>P.18</t>
+          <t>R.3</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Export' icon to initiate the export process and trigger the file download.</t>
+          <t>Close the browser context to clean up resources and end the session.</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`context.close()`</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr"/>
@@ -2896,336 +3078,26 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>P.19</t>
+          <t>R.4</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Click on the second page link in the pagination to navigate to the second page of the grid.</t>
+          <t>Close the browser instance to terminate all associated contexts and sessions.</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("a").nth(2).click()`</t>
+          <t>`browser.close()`</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr"/>
       <c r="E132" s="4" t="inlineStr"/>
       <c r="F132" s="4" t="inlineStr"/>
     </row>
-    <row r="133">
-      <c r="A133" s="3" t="inlineStr">
-        <is>
-          <t>P.20</t>
-        </is>
-      </c>
-      <c r="B133" s="4" t="inlineStr">
-        <is>
-          <t>Click on the page link labeled '3' to navigate to the third page of the grid.</t>
-        </is>
-      </c>
-      <c r="C133" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("a").filter(has_text="3").click()`</t>
-        </is>
-      </c>
-      <c r="D133" s="3" t="inlineStr"/>
-      <c r="E133" s="4" t="inlineStr"/>
-      <c r="F133" s="4" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" s="3" t="inlineStr">
-        <is>
-          <t>P.21</t>
-        </is>
-      </c>
-      <c r="B134" s="4" t="inlineStr">
-        <is>
-          <t>Click on the 'First Page' button in the pagination controls to navigate back to the first page of the grid.</t>
-        </is>
-      </c>
-      <c r="C134" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .card-content &gt; esp-row-dimentional-grid &gt; div &gt; #paginationId &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first").click()`</t>
-        </is>
-      </c>
-      <c r="D134" s="3" t="inlineStr"/>
-      <c r="E134" s="4" t="inlineStr"/>
-      <c r="F134" s="4" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="inlineStr">
-        <is>
-          <t>--- ROW DISPLAY AND COLUMN FILTERING ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="3" t="inlineStr">
-        <is>
-          <t>Q.1</t>
-        </is>
-      </c>
-      <c r="B136" s="4" t="inlineStr">
-        <is>
-          <t>Click on the dropdown labeled 'View 10 row(s)' to open the row display options.</t>
-        </is>
-      </c>
-      <c r="C136" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_text("View 10 row(s)").nth(2).click()`</t>
-        </is>
-      </c>
-      <c r="D136" s="3" t="inlineStr"/>
-      <c r="E136" s="4" t="inlineStr"/>
-      <c r="F136" s="4" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="3" t="inlineStr">
-        <is>
-          <t>Q.2</t>
-        </is>
-      </c>
-      <c r="B137" s="4" t="inlineStr">
-        <is>
-          <t>Select the option 'View 20 row(s)' from the dropdown to change the number of rows displayed.</t>
-        </is>
-      </c>
-      <c r="C137" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^View 20 row\(s\)$")).nth(1).click()`</t>
-        </is>
-      </c>
-      <c r="D137" s="3" t="inlineStr"/>
-      <c r="E137" s="4" t="inlineStr"/>
-      <c r="F137" s="4" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" s="3" t="inlineStr">
-        <is>
-          <t>Q.3</t>
-        </is>
-      </c>
-      <c r="B138" s="4" t="inlineStr">
-        <is>
-          <t>Click on the column header icon to open the filter options for the column.</t>
-        </is>
-      </c>
-      <c r="C138" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
-        </is>
-      </c>
-      <c r="D138" s="3" t="inlineStr"/>
-      <c r="E138" s="4" t="inlineStr"/>
-      <c r="F138" s="4" t="inlineStr"/>
-    </row>
-    <row r="139">
-      <c r="A139" s="3" t="inlineStr">
-        <is>
-          <t>Q.4</t>
-        </is>
-      </c>
-      <c r="B139" s="4" t="inlineStr">
-        <is>
-          <t>Fill the filter textbox with the value 'Promotion' to filter the column based on this value.</t>
-        </is>
-      </c>
-      <c r="C139" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("textbox", name="Filter Value").fill("Promotion")`</t>
-        </is>
-      </c>
-      <c r="D139" s="3" t="inlineStr"/>
-      <c r="E139" s="4" t="inlineStr"/>
-      <c r="F139" s="4" t="inlineStr"/>
-    </row>
-    <row r="140">
-      <c r="A140" s="3" t="inlineStr">
-        <is>
-          <t>Q.5</t>
-        </is>
-      </c>
-      <c r="B140" s="4" t="inlineStr">
-        <is>
-          <t>Click the 'Apply' button to apply the column filter.</t>
-        </is>
-      </c>
-      <c r="C140" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
-        </is>
-      </c>
-      <c r="D140" s="3" t="inlineStr"/>
-      <c r="E140" s="4" t="inlineStr"/>
-      <c r="F140" s="4" t="inlineStr"/>
-    </row>
-    <row r="141">
-      <c r="A141" s="3" t="inlineStr">
-        <is>
-          <t>Q.6</t>
-        </is>
-      </c>
-      <c r="B141" s="4" t="inlineStr">
-        <is>
-          <t>Click on the filtered column header to interact with the column filter settings.</t>
-        </is>
-      </c>
-      <c r="C141" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-cell-filtered &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container").click()`</t>
-        </is>
-      </c>
-      <c r="D141" s="3" t="inlineStr"/>
-      <c r="E141" s="4" t="inlineStr"/>
-      <c r="F141" s="4" t="inlineStr"/>
-    </row>
-    <row r="142">
-      <c r="A142" s="3" t="inlineStr">
-        <is>
-          <t>Q.7</t>
-        </is>
-      </c>
-      <c r="B142" s="4" t="inlineStr">
-        <is>
-          <t>Click on the filter icon to open the active filter options for the column.</t>
-        </is>
-      </c>
-      <c r="C142" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
-        </is>
-      </c>
-      <c r="D142" s="3" t="inlineStr"/>
-      <c r="E142" s="4" t="inlineStr"/>
-      <c r="F142" s="4" t="inlineStr"/>
-    </row>
-    <row r="143">
-      <c r="A143" s="3" t="inlineStr">
-        <is>
-          <t>Q.8</t>
-        </is>
-      </c>
-      <c r="B143" s="4" t="inlineStr">
-        <is>
-          <t>Click the 'Reset' button to clear the applied column filter.</t>
-        </is>
-      </c>
-      <c r="C143" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
-        </is>
-      </c>
-      <c r="D143" s="3" t="inlineStr"/>
-      <c r="E143" s="4" t="inlineStr"/>
-      <c r="F143" s="4" t="inlineStr"/>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="inlineStr">
-        <is>
-          <t>--- FINAL GRID INTERACTIONS AND CLEANUP ---</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="3" t="inlineStr">
-        <is>
-          <t>R.1</t>
-        </is>
-      </c>
-      <c r="B145" s="4" t="inlineStr">
-        <is>
-          <t>Double-click on the grid cell with the name 'Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/' to interact with or edit the cell.</t>
-        </is>
-      </c>
-      <c r="C145" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("gridcell", name="Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/").dblclick()`</t>
-        </is>
-      </c>
-      <c r="D145" s="3" t="inlineStr"/>
-      <c r="E145" s="4" t="inlineStr"/>
-      <c r="F145" s="4" t="inlineStr"/>
-    </row>
-    <row r="146">
-      <c r="A146" s="3" t="inlineStr">
-        <is>
-          <t>R.2</t>
-        </is>
-      </c>
-      <c r="B146" s="4" t="inlineStr">
-        <is>
-          <t>Close the current page after completing the interaction.</t>
-        </is>
-      </c>
-      <c r="C146" s="4" t="inlineStr">
-        <is>
-          <t>`page.close()`</t>
-        </is>
-      </c>
-      <c r="D146" s="3" t="inlineStr"/>
-      <c r="E146" s="4" t="inlineStr"/>
-      <c r="F146" s="4" t="inlineStr"/>
-    </row>
-    <row r="147">
-      <c r="A147" s="3" t="inlineStr">
-        <is>
-          <t>R.3</t>
-        </is>
-      </c>
-      <c r="B147" s="4" t="inlineStr">
-        <is>
-          <t>Close the browser context to clean up resources and end the session.</t>
-        </is>
-      </c>
-      <c r="C147" s="4" t="inlineStr">
-        <is>
-          <t>`context.close()`</t>
-        </is>
-      </c>
-      <c r="D147" s="3" t="inlineStr"/>
-      <c r="E147" s="4" t="inlineStr"/>
-      <c r="F147" s="4" t="inlineStr"/>
-    </row>
-    <row r="148">
-      <c r="A148" s="3" t="inlineStr">
-        <is>
-          <t>R.4</t>
-        </is>
-      </c>
-      <c r="B148" s="4" t="inlineStr">
-        <is>
-          <t>Close the browser instance to terminate all associated contexts and sessions.</t>
-        </is>
-      </c>
-      <c r="C148" s="4" t="inlineStr">
-        <is>
-          <t>`browser.close()`</t>
-        </is>
-      </c>
-      <c r="D148" s="3" t="inlineStr"/>
-      <c r="E148" s="4" t="inlineStr"/>
-      <c r="F148" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A41:F41"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="A92:F92"/>
-    <mergeCell ref="A113:F113"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A75:F75"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A103:F103"/>
-    <mergeCell ref="A144:F144"/>
-    <mergeCell ref="A135:F135"/>
-    <mergeCell ref="A83:F83"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fixed ag playback issues
</commit_message>
<xml_diff>
--- a/UAT_Excel_Reports/Bbu Alerts_UAT.xlsx
+++ b/UAT_Excel_Reports/Bbu Alerts_UAT.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -496,39 +496,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>C.1</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Navigate to the 'Executive Dashboard' in the demand planning application by entering the specified URL in the browser.</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>`page.goto("https://stage.bbu.esp.antuit.ai/dp/demand-planning/executive-dashboard?workbookId=4&amp;tabIndex=1")`</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>--- INITIAL NAVIGATION TO DASHBOARD ---</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>D.1</t>
+          <t>C.1</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter' button to open the filter options in the dashboard.</t>
+          <t>Navigate to the 'Executive Dashboard' in the demand planning application by entering the specified URL in the browser.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Filter").click()`</t>
+          <t>`page.goto("https://stage.bbu.esp.antuit.ai/dp/demand-planning/executive-dashboard?workbookId=4&amp;tabIndex=1")`</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr"/>
@@ -536,39 +523,26 @@
       <c r="F4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>D.2</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>From the filter dropdown, select the 'Alerts' option to filter by alerts.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("#alerts-filterId").get_by_text("Alerts").click()`</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>--- FILTER INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>D.3</t>
+          <t>D.1</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret to expand the filter options.</t>
+          <t>Click on the 'Filter' button to open the filter options in the dashboard.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".dropdown-caret").first.click()`</t>
+          <t>`page.get_by_text("Filter").click()`</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr"/>
@@ -578,17 +552,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>D.4</t>
+          <t>D.2</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Over Bias' filter option.</t>
+          <t>From the filter dropdown, select the 'Alerts' option to filter by alerts.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Over Bias$")).nth(1).click()`</t>
+          <t>`page.locator("#alerts-filterId").get_by_text("Alerts").click()`</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
@@ -598,12 +572,12 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>D.5</t>
+          <t>D.3</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to expand the filter options.</t>
+          <t>Click on the dropdown caret to expand the filter options.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -618,17 +592,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>D.6</t>
+          <t>D.4</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Under Bias' filter option.</t>
+          <t>From the expanded dropdown, select the 'Over Bias' filter option.</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Under Bias$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Over Bias$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
@@ -638,7 +612,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>D.7</t>
+          <t>D.5</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -658,17 +632,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>D.8</t>
+          <t>D.6</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'MAPE' filter option.</t>
+          <t>From the expanded dropdown, select the 'Under Bias' filter option.</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^MAPE$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Under Bias$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr"/>
@@ -678,7 +652,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>D.9</t>
+          <t>D.7</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -698,17 +672,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>D.10</t>
+          <t>D.8</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'Stability' filter option.</t>
+          <t>From the expanded dropdown, select the 'MAPE' filter option.</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Stability$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^MAPE$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
@@ -718,7 +692,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>D.11</t>
+          <t>D.9</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -738,17 +712,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>D.12</t>
+          <t>D.10</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>From the expanded dropdown, select the 'FVA' filter option.</t>
+          <t>From the expanded dropdown, select the 'Stability' filter option.</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^FVA$")).nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Stability$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr"/>
@@ -758,17 +732,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>E.1</t>
+          <t>D.11</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
+          <t>Click on the dropdown caret again to expand the filter options.</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").click()`</t>
+          <t>`page.locator(".dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr"/>
@@ -778,17 +752,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>E.2</t>
+          <t>D.12</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>From the expanded dropdown, select the 'FVA' filter option.</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^FVA$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr"/>
@@ -796,39 +770,26 @@
       <c r="F17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>E.3</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Uncheck the '6W-Actuals Column' checkbox to hide this specific column.</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("treeitem", name="6W-Actuals Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>--- COLUMN VISIBILITY CONFIGURATION ---</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>E.4</t>
+          <t>E.1</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the 'User Bias Column' checkbox to hide this specific column.</t>
+          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="User Bias Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("button", name="columns").click()`</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
@@ -838,17 +799,17 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>F.1</t>
+          <t>E.2</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Adjustments' button to open the preferences menu.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr"/>
@@ -858,17 +819,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>F.2</t>
+          <t>E.3</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
+          <t>Uncheck the '6W-Actuals Column' checkbox to hide this specific column.</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.get_by_role("treeitem", name="6W-Actuals Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr"/>
@@ -878,17 +839,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>F.3</t>
+          <t>E.4</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Download' button to export the saved preferences.</t>
+          <t>Uncheck the 'User Bias Column' checkbox to hide this specific column.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".icon-color-toolbar-active.zeb-download-underline").click()`</t>
+          <t>`page.get_by_role("treeitem", name="User Bias Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
@@ -896,39 +857,26 @@
       <c r="F22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>G.1</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Click on the 'Adjustments' button again to reopen the preferences menu.</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>--- PREFERENCES AND DOWNLOAD HANDLING ---</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>G.2</t>
+          <t>F.1</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Reset Preference' to revert to the default column visibility settings.</t>
+          <t>Click on the 'Adjustments' button to open the preferences menu.</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr"/>
@@ -938,17 +886,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>G.3</t>
+          <t>F.2</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon to open the filter menu for the first column.</t>
+          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr"/>
@@ -958,17 +906,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>G.4</t>
+          <t>F.3</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Enter 'WINCO' into the filter text box to filter the data by this value.</t>
+          <t>Click on the 'Download' button to export the saved preferences.</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Value").fill("WINCO")`</t>
+          <t>`page.locator(".icon-color-toolbar-active.zeb-download-underline").click()`</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr"/>
@@ -976,39 +924,26 @@
       <c r="F26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>G.5</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Click on the 'Apply' button to apply the filter and update the data view.</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("button", name="Apply").click()`</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>--- FILTER AND STATUS DROPDOWN INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>G.6</t>
+          <t>G.1</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon again to reopen the filter menu for the first column.</t>
+          <t>Click on the 'Adjustments' button again to reopen the preferences menu.</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
+          <t>`page.locator(".pointer.zeb-adjustments").click()`</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr"/>
@@ -1018,17 +953,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>G.7</t>
+          <t>G.2</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset' button to clear the applied filter and restore the default data view.</t>
+          <t>Click on 'Reset Preference' to revert to the default column visibility settings.</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="Reset").click()`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr"/>
@@ -1038,17 +973,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>G.8</t>
+          <t>G.3</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret to open the dropdown menu for selecting a status.</t>
+          <t>Click on the filter icon to open the filter menu for the first column.</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr"/>
@@ -1058,17 +993,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>G.9</t>
+          <t>G.4</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Select the 'In progress' option from the dropdown menu.</t>
+          <t>Enter 'WINCO' into the filter text box to filter the data by this value.</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("In progress").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Value").fill("WINCO")`</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr"/>
@@ -1078,17 +1013,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>G.10</t>
+          <t>G.5</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
+          <t>Click on the 'Apply' button to apply the filter and update the data view.</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.get_by_role("button", name="Apply").click()`</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr"/>
@@ -1098,17 +1033,17 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>G.11</t>
+          <t>G.6</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Completed' option from the dropdown menu.</t>
+          <t>Click on the filter icon again to reopen the filter menu for the first column.</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Completed").click()`</t>
+          <t>`page.locator(".ag-icon.ag-icon-filter").first.click()`</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr"/>
@@ -1118,17 +1053,17 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>G.12</t>
+          <t>G.7</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
+          <t>Click on the 'Reset' button to clear the applied filter and restore the default data view.</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
+          <t>`page.get_by_role("button", name="Reset").click()`</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr"/>
@@ -1138,17 +1073,17 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>G.13</t>
+          <t>G.8</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Not started' option from the dropdown menu.</t>
+          <t>Click on the dropdown caret to open the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Not started").click()`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr"/>
@@ -1158,17 +1093,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>H.1</t>
+          <t>G.9</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Double-click on 'WALMART STORES HQ' in the treegrid to expand its details.</t>
+          <t>Select the 'In progress' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").dblclick()`</t>
+          <t>`page.get_by_text("In progress").click()`</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr"/>
@@ -1178,17 +1113,17 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>H.2</t>
+          <t>G.10</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the first occurrence of the text 'WALMART' to navigate further.</t>
+          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("span").filter(has_text="WALMART").first.dblclick()`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr"/>
@@ -1198,17 +1133,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>H.3</t>
+          <t>G.11</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Double-click on 'WALMART 0906 SC B-0006805-01-' in the treegrid to expand its details.</t>
+          <t>Select the 'Completed' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART 0906 SC B-0006805-01-").dblclick()`</t>
+          <t>`page.get_by_text("Completed").click()`</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr"/>
@@ -1218,17 +1153,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>H.4</t>
+          <t>G.12</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Right-click on 'WALMART 0906 SC B-0006805-01-' to open the context menu.</t>
+          <t>Click on the dropdown caret again to reopen the dropdown menu for selecting a status.</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("WALMART 0906 SC B-0006805-01-").click(button="right")`</t>
+          <t>`page.locator(".w-100.p-h-16.p-v-8.dropdown-label.icon-small-dropdown &gt; .d-flex.align-items-center &gt; .dropdown-caret").first.click()`</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr"/>
@@ -1238,17 +1173,17 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>H.5</t>
+          <t>G.13</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Select the 'Not started' option from the dropdown menu.</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.get_by_text("Not started").click()`</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr"/>
@@ -1256,39 +1191,26 @@
       <c r="F40" s="4" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>H.6</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Right-click on the highlighted row in the treegrid to open the context menu.</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".ag-row-even.ag-row-focus.ag-row-not-inline-editing.ag-row.ag-row-level-0.ag-row-position-absolute.ag-row-first.ag-row-hover &gt; .ag-cell-value &gt; .ag-cell-wrapper").click(button="right")`</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr"/>
-      <c r="E41" s="4" t="inlineStr"/>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>--- TREEGRID INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>H.7</t>
+          <t>H.1</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Double-click on 'WALMART STORES HQ' in the treegrid to expand its details.</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").dblclick()`</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr"/>
@@ -1298,17 +1220,17 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>H.8</t>
+          <t>H.2</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Right-click on 'WALMART STORES HQ' in the treegrid to open the context menu.</t>
+          <t>Double-click on the first occurrence of the text 'WALMART' to navigate further.</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").click(button="right")`</t>
+          <t>`page.locator("span").filter(has_text="WALMART").first.dblclick()`</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr"/>
@@ -1318,17 +1240,17 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>H.9</t>
+          <t>H.3</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
+          <t>Double-click on 'WALMART 0906 SC B-0006805-01-' in the treegrid to expand its details.</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART 0906 SC B-0006805-01-").dblclick()`</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr"/>
@@ -1338,17 +1260,17 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>I.1</t>
+          <t>H.4</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Click on the column header labeled '6W-Actuals' to sort or interact with the column.</t>
+          <t>Right-click on 'WALMART 0906 SC B-0006805-01-' to open the context menu.</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("columnheader", name="6W-Actuals").click()`</t>
+          <t>`page.get_by_text("WALMART 0906 SC B-0006805-01-").click(button="right")`</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr"/>
@@ -1358,17 +1280,17 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>I.2</t>
+          <t>H.5</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Click on the page number '2' in the pagination control to navigate to the second page of the grid.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("a").filter(has_text="2").click()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr"/>
@@ -1378,17 +1300,17 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>I.3</t>
+          <t>H.6</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'First Page' button in the pagination control to navigate to the first page of the grid.</t>
+          <t>Right-click on the highlighted row in the treegrid to open the context menu.</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".zeb-nav-to-first").click()`</t>
+          <t>`page.locator(".ag-row-even.ag-row-focus.ag-row-not-inline-editing.ag-row.ag-row-level-0.ag-row-position-absolute.ag-row-first.ag-row-hover &gt; .ag-cell-value &gt; .ag-cell-wrapper").click(button="right")`</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr"/>
@@ -1398,17 +1320,17 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>I.4</t>
+          <t>H.7</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Select the row containing 'WALMART STORES HQ' by checking the checkbox in the grid cell.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell", name="Press Space to toggle row selection (unchecked)   WALMART STORES HQ").get_by_label("Press Space to toggle row").check()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr"/>
@@ -1418,17 +1340,17 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>I.5</t>
+          <t>H.8</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
+          <t>Right-click on 'WALMART STORES HQ' in the treegrid to open the context menu.</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.uncheck()`</t>
+          <t>`page.get_by_role("treegrid").get_by_text("WALMART STORES HQ").click(button="right")`</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr"/>
@@ -1438,17 +1360,17 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>I.6</t>
+          <t>H.9</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Check the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
+          <t>Click on 'Drill up' from the context menu to navigate up one level.</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
@@ -1456,39 +1378,26 @@
       <c r="F50" s="4" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>I.7</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Uncheck the first checkbox in the grid using the '.d-flex.align-items-center.checkbox-primary-color' locator.</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".d-flex.align-items-center.checkbox-primary-color").first.uncheck()`</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="4" t="inlineStr"/>
-      <c r="F51" s="4" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>--- PAGINATION AND GRID INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>I.8</t>
+          <t>I.1</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the first checkbox in the grid using a more specific locator targeting a nested structure within the grid.</t>
+          <t>Click on the column header labeled '6W-Actuals' to sort or interact with the column.</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-row-odd &gt; .ag-cell-value &gt; .ag-cell-wrapper &gt; .ag-group-value &gt; aeap-group-cell-renderer &gt; .d-flex.align-items-center.w-fit-content &gt; .d-flex").first.uncheck()`</t>
+          <t>`page.get_by_role("columnheader", name="6W-Actuals").click()`</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr"/>
@@ -1498,17 +1407,17 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>J.1</t>
+          <t>I.2</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
+          <t>Click on the page number '2' in the pagination control to navigate to the second page of the grid.</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
+          <t>`page.locator("a").filter(has_text="2").click()`</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr"/>
@@ -1518,17 +1427,17 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>J.2</t>
+          <t>I.3</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>Click on the 'First Page' button in the pagination control to navigate to the first page of the grid.</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.locator(".zeb-nav-to-first").click()`</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr"/>
@@ -1538,17 +1447,17 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>J.3</t>
+          <t>I.4</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
+          <t>Select the row containing 'WALMART STORES HQ' by checking the checkbox in the grid cell.</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.get_by_role("gridcell", name="Press Space to toggle row selection (unchecked)   WALMART STORES HQ").get_by_label("Press Space to toggle row").check()`</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr"/>
@@ -1558,17 +1467,17 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>J.4</t>
+          <t>I.5</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Fill the 'Filter Columns Input' textbox with the text 'User Bias' to filter columns by this keyword.</t>
+          <t>Uncheck the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("User Bias")`</t>
+          <t>`page.locator(".checkbox-primary-color").first.uncheck()`</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr"/>
@@ -1578,17 +1487,17 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>J.5</t>
+          <t>I.6</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the checkbox corresponding to the 'User Bias' column to hide it.</t>
+          <t>Check the first checkbox in the grid using the '.checkbox-primary-color' locator.</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr"/>
@@ -1598,17 +1507,17 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>J.6</t>
+          <t>I.7</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox again to focus on it.</t>
+          <t>Uncheck the first checkbox in the grid using the '.d-flex.align-items-center.checkbox-primary-color' locator.</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.locator(".d-flex.align-items-center.checkbox-primary-color").first.uncheck()`</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr"/>
@@ -1618,17 +1527,17 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>J.7</t>
+          <t>I.8</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>Select all text in the 'Filter Columns Input' textbox using the 'ControlOrMeta+a' keyboard shortcut.</t>
+          <t>Uncheck the first checkbox in the grid using a more specific locator targeting a nested structure within the grid.</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").press("ControlOrMeta+a")`</t>
+          <t>`page.locator(".ag-row-odd &gt; .ag-cell-value &gt; .ag-cell-wrapper &gt; .ag-group-value &gt; aeap-group-cell-renderer &gt; .d-flex.align-items-center.w-fit-content &gt; .d-flex").first.uncheck()`</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr"/>
@@ -1636,39 +1545,26 @@
       <c r="F59" s="4" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>J.8</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>Clear the 'Filter Columns Input' textbox by filling it with an empty string.</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("")`</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr"/>
-      <c r="E60" s="4" t="inlineStr"/>
-      <c r="F60" s="4" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>--- ADVANCED COLUMN VISIBILITY CONFIGURATION ---</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>J.9</t>
+          <t>J.1</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox again to ensure all columns are visible.</t>
+          <t>Click on the 'Columns' button to open the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr"/>
@@ -1678,17 +1574,17 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>J.10</t>
+          <t>J.2</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Columns' button to close the column visibility configuration panel.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr"/>
@@ -1698,17 +1594,17 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>K.1</t>
+          <t>J.3</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' dropdown menu to open the preference options.</t>
+          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr"/>
@@ -1718,17 +1614,17 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>K.2</t>
+          <t>J.4</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Save Preference' option to save the current grid settings.</t>
+          <t>Fill the 'Filter Columns Input' textbox with the text 'User Bias' to filter columns by this keyword.</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("User Bias")`</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr"/>
@@ -1738,17 +1634,17 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>K.3</t>
+          <t>J.5</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Export' button to export the grid data, triggering a file download.</t>
+          <t>Uncheck the checkbox corresponding to the 'User Bias' column to hide it.</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(2) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr"/>
@@ -1758,17 +1654,17 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>L.1</t>
+          <t>J.6</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' dropdown menu again to reopen the preference options.</t>
+          <t>Click on the 'Filter Columns Input' textbox again to focus on it.</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr"/>
@@ -1778,17 +1674,17 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>L.2</t>
+          <t>J.7</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset Preference' option to revert the grid settings to their default state.</t>
+          <t>Select all text in the 'Filter Columns Input' textbox using the 'ControlOrMeta+a' keyboard shortcut.</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").press("ControlOrMeta+a")`</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr"/>
@@ -1798,17 +1694,17 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>L.3</t>
+          <t>J.8</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon in the column header to open the filter options for the selected column.</t>
+          <t>Clear the 'Filter Columns Input' textbox by filling it with an empty string.</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("")`</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr"/>
@@ -1818,17 +1714,17 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>L.4</t>
+          <t>J.9</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Enter the filter value '761' into the filter input field to apply a filter to the column.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox again to ensure all columns are visible.</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("spinbutton", name="Filter Value").fill("761")`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr"/>
@@ -1838,17 +1734,17 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>L.5</t>
+          <t>J.10</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Apply' button in the column filter menu to apply the filter and update the grid data.</t>
+          <t>Click on the 'Columns' button to close the column visibility configuration panel.</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
+          <t>`page.get_by_role("button", name="columns").nth(1).click()`</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr"/>
@@ -1856,39 +1752,26 @@
       <c r="F70" s="4" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>L.6</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>Click on the filter icon again to reopen the column filter menu after applying the filter.</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="4" t="inlineStr"/>
-      <c r="F71" s="4" t="inlineStr"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>--- PREFERENCE AND EXPORT HANDLING ---</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>L.7</t>
+          <t>K.1</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Reset' button in the column filter menu to clear the applied filter and restore the grid data to its original state.</t>
+          <t>Click on the 'Preference' dropdown menu to open the preference options.</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr"/>
@@ -1898,17 +1781,17 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>M.1</t>
+          <t>K.2</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Check the first checkbox with the primary color styling to select the corresponding row.</t>
+          <t>Click on the 'Save Preference' option to save the current grid settings.</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr"/>
@@ -1918,17 +1801,17 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>M.2</t>
+          <t>K.3</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the row containing the text 'ENTENMANNS' to drill down into its details.</t>
+          <t>Click on the 'Export' button to export the grid data, triggering a file download.</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("span").filter(has_text="ENTENMANNS").first.dblclick()`</t>
+          <t>`page.locator("div:nth-child(2) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr"/>
@@ -1936,39 +1819,26 @@
       <c r="F74" s="4" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>M.3</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>Double-click on the row containing the text 'EN BITES' to further drill down into its details.</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("span").filter(has_text="EN BITES").first.dblclick()`</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr"/>
-      <c r="E75" s="4" t="inlineStr"/>
-      <c r="F75" s="4" t="inlineStr"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>--- COLUMN FILTERING AND RESET ---</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>M.4</t>
+          <t>L.1</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the row containing the text 'EN LITTLE BITES CP' to navigate deeper into its details.</t>
+          <t>Click on the 'Preference' dropdown menu again to reopen the preference options.</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("EN LITTLE BITES CP").first.dblclick()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr"/>
@@ -1978,17 +1848,17 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>M.5</t>
+          <t>L.2</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Right-click on the row containing the text 'EN LB CHOCCH MFN 10P-' to open the context menu for additional actions.</t>
+          <t>Click on the 'Reset Preference' option to revert the grid settings to their default state.</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("EN LB CHOCCH MFN 10P-").first.click(button="right")`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr"/>
@@ -1998,17 +1868,17 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>M.6</t>
+          <t>L.3</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Drill up' option in the context menu to navigate back to the previous level.</t>
+          <t>Click on the filter icon in the column header to open the filter options for the selected column.</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Drill up").click()`</t>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr"/>
@@ -2018,17 +1888,17 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>M.7</t>
+          <t>L.4</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Right-click on the first grid cell with an empty text value to open the context menu.</t>
+          <t>Enter the filter value '761' into the filter input field to apply a filter to the column.</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click(button="right")`</t>
+          <t>`page.get_by_role("spinbutton", name="Filter Value").fill("761")`</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr"/>
@@ -2038,17 +1908,17 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>M.8</t>
+          <t>L.5</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Click on the first grid cell with an empty text value to select it.</t>
+          <t>Click on the 'Apply' button in the column filter menu to apply the filter and update the grid data.</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr"/>
@@ -2058,17 +1928,17 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>N.1</t>
+          <t>L.6</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Click on the link within the 'Products' card to navigate to the detailed view of the products.</t>
+          <t>Click on the filter icon again to reopen the column filter menu after applying the filter.</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Products10 rows out of 11").locator("a").click()`</t>
+          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr"/>
@@ -2078,17 +1948,17 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>N.2</t>
+          <t>L.7</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'First Page' button in the pagination controls to navigate to the first page of the product list.</t>
+          <t>Click on the 'Reset' button in the column filter menu to clear the applied filter and restore the grid data to its original state.</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first &gt; .zeb-nav-to-first").click()`</t>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr"/>
@@ -2096,39 +1966,26 @@
       <c r="F82" s="4" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="3" t="inlineStr">
-        <is>
-          <t>N.3</t>
-        </is>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Click on the 'Apply' button to apply the selected filters or changes.</t>
-        </is>
-      </c>
-      <c r="C83" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("button", name="Apply").click()`</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr"/>
-      <c r="E83" s="4" t="inlineStr"/>
-      <c r="F83" s="4" t="inlineStr"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>--- ROW AND DRILL-DOWN INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>N.4</t>
+          <t>M.1</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter' section to expand or interact with the filter options.</t>
+          <t>Check the first checkbox with the primary color styling to select the corresponding row.</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Filter$")).nth(1).click()`</t>
+          <t>`page.locator(".checkbox-primary-color").first.check()`</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr"/>
@@ -2138,17 +1995,17 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>N.5</t>
+          <t>M.2</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter to open the dropdown menu.</t>
+          <t>Double-click on the row containing the text 'ENTENMANNS' to drill down into its details.</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.locator("span").filter(has_text="ENTENMANNS").first.dblclick()`</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr"/>
@@ -2158,17 +2015,17 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>N.6</t>
+          <t>M.3</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 5 Next 4' option from the 'Time' filter dropdown.</t>
+          <t>Double-click on the row containing the text 'EN BITES' to further drill down into its details.</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 4$")).nth(1).click()`</t>
+          <t>`page.locator("span").filter(has_text="EN BITES").first.dblclick()`</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr"/>
@@ -2178,17 +2035,17 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>N.7</t>
+          <t>M.4</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for a new selection.</t>
+          <t>Double-click on the row containing the text 'EN LITTLE BITES CP' to navigate deeper into its details.</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.get_by_text("EN LITTLE BITES CP").first.dblclick()`</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr"/>
@@ -2198,17 +2055,17 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>N.8</t>
+          <t>M.5</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 5 Next 12' option from the 'Time' filter dropdown.</t>
+          <t>Right-click on the row containing the text 'EN LB CHOCCH MFN 10P-' to open the context menu for additional actions.</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 12$")).nth(1).click()`</t>
+          <t>`page.get_by_text("EN LB CHOCCH MFN 10P-").first.click(button="right")`</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr"/>
@@ -2218,17 +2075,17 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>N.9</t>
+          <t>M.6</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for another selection.</t>
+          <t>Click on the 'Drill up' option in the context menu to navigate back to the previous level.</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
+          <t>`page.get_by_text("Drill up").click()`</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr"/>
@@ -2238,17 +2095,17 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>N.10</t>
+          <t>M.7</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Select the 'Latest 13 Next 4' option from the 'Time' filter dropdown.</t>
+          <t>Right-click on the first grid cell with an empty text value to open the context menu.</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 13 Next 4$")).nth(1).click()`</t>
+          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click(button="right")`</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr"/>
@@ -2258,17 +2115,17 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>O.1</t>
+          <t>M.8</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Weekly Summary Customer:' card button to expand or interact with the card.</t>
+          <t>Click on the first grid cell with an empty text value to select it.</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Weekly Summary Customer:").get_by_role("button").click()`</t>
+          <t>`page.get_by_role("gridcell").filter(has_text=re.compile(r"^$")).first.click()`</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr"/>
@@ -2276,39 +2133,26 @@
       <c r="F91" s="4" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>O.2</t>
-        </is>
-      </c>
-      <c r="B92" s="4" t="inlineStr">
-        <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-02 (45) Column'.</t>
-        </is>
-      </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("treeitem", name="-11-02 (45) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
-        </is>
-      </c>
-      <c r="D92" s="3" t="inlineStr"/>
-      <c r="E92" s="4" t="inlineStr"/>
-      <c r="F92" s="4" t="inlineStr"/>
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>--- PRODUCT NAVIGATION AND TIME FILTER ---</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>O.3</t>
+          <t>N.1</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-09 (46) Column'.</t>
+          <t>Click on the link within the 'Products' card to navigate to the detailed view of the products.</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="-11-09 (46) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("esp-card-component").filter(has_text="Products10 rows out of 11").locator("a").click()`</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr"/>
@@ -2318,17 +2162,17 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>O.4</t>
+          <t>N.2</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the column labeled '-11-16 (47) Column'.</t>
+          <t>Click on the 'First Page' button in the pagination controls to navigate to the first page of the product list.</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="-11-16 (47) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first &gt; .zeb-nav-to-first").click()`</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr"/>
@@ -2338,17 +2182,17 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>O.5</t>
+          <t>N.3</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
+          <t>Click on the 'Apply' button to apply the selected filters or changes.</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.get_by_role("button", name="Apply").click()`</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr"/>
@@ -2358,17 +2202,17 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>O.6</t>
+          <t>N.4</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Click on the preference dropdown icon to open the preference options.</t>
+          <t>Click on the 'Filter' section to expand or interact with the filter options.</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Filter$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr"/>
@@ -2378,17 +2222,17 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>O.7</t>
+          <t>N.5</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
+          <t>Click on the dropdown caret in the 'Time' filter to open the dropdown menu.</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr"/>
@@ -2398,17 +2242,17 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>O.8</t>
+          <t>N.6</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Click on the preference dropdown icon again to reopen the preference options.</t>
+          <t>Select the 'Latest 5 Next 4' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 4$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr"/>
@@ -2418,17 +2262,17 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>O.9</t>
+          <t>N.7</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Reset Preference' to reset the column visibility settings to their default state.</t>
+          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for a new selection.</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Reset Preference").click()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr"/>
@@ -2438,17 +2282,17 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>P.1</t>
+          <t>N.8</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Click on the export icon to initiate the download process.</t>
+          <t>Select the 'Latest 5 Next 12' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(3) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 5 Next 12$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr"/>
@@ -2458,17 +2302,17 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>P.2</t>
+          <t>N.9</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Click on the first element with the class 'align-middle' to interact with it.</t>
+          <t>Click on the dropdown caret in the 'Time' filter again to open the dropdown menu for another selection.</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".align-middle").first.click()`</t>
+          <t>`page.locator("#time-filterId &gt; .wr-20 &gt; esp-multiselect-dropdown &gt; .multiselect-dropdown &gt; div &gt; .w-100 &gt; .d-flex.align-items-center &gt; .dropdown-caret").click()`</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr"/>
@@ -2478,17 +2322,17 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>P.3</t>
+          <t>N.10</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Click on the second occurrence of the text 'Event' to navigate or interact with the Event section.</t>
+          <t>Select the 'Latest 13 Next 4' option from the 'Time' filter dropdown.</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Event").nth(1).click()`</t>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^Latest 13 Next 4$")).nth(1).click()`</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr"/>
@@ -2496,39 +2340,26 @@
       <c r="F102" s="4" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="3" t="inlineStr">
-        <is>
-          <t>P.4</t>
-        </is>
-      </c>
-      <c r="B103" s="4" t="inlineStr">
-        <is>
-          <t>Click on the button within the 'Event Details columns (0)' card to open column visibility options.</t>
-        </is>
-      </c>
-      <c r="C103" s="4" t="inlineStr">
-        <is>
-          <t>`page.locator("esp-card-component").filter(has_text="Event Details columns (0)").get_by_role("button").click()`</t>
-        </is>
-      </c>
-      <c r="D103" s="3" t="inlineStr"/>
-      <c r="E103" s="4" t="inlineStr"/>
-      <c r="F103" s="4" t="inlineStr"/>
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>--- WEEKLY SUMMARY AND COLUMN VISIBILITY ---</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>P.5</t>
+          <t>O.1</t>
         </is>
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Event Column' to hide it.</t>
+          <t>Click on the 'Weekly Summary Customer:' card button to expand or interact with the card.</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Event Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("esp-card-component").filter(has_text="Weekly Summary Customer:").get_by_role("button").click()`</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr"/>
@@ -2538,17 +2369,17 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>P.6</t>
+          <t>O.2</t>
         </is>
       </c>
       <c r="B105" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'UPC 12 Column' to hide it.</t>
+          <t>Uncheck the visibility toggle for the column labeled '-11-02 (45) Column'.</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="UPC 12 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="-11-02 (45) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr"/>
@@ -2558,17 +2389,17 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>P.7</t>
+          <t>O.3</t>
         </is>
       </c>
       <c r="B106" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Customer Level 2 Column' to hide it.</t>
+          <t>Uncheck the visibility toggle for the column labeled '-11-09 (46) Column'.</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Customer Level 2 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="-11-09 (46) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr"/>
@@ -2578,17 +2409,17 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>P.8</t>
+          <t>O.4</t>
         </is>
       </c>
       <c r="B107" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Start Date Column' to hide it.</t>
+          <t>Uncheck the visibility toggle for the column labeled '-11-16 (47) Column'.</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Start Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("treeitem", name="-11-16 (47) Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr"/>
@@ -2598,17 +2429,17 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>P.9</t>
+          <t>O.5</t>
         </is>
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'End Date Column' to hide it.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible.</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="End Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr"/>
@@ -2618,17 +2449,17 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>P.10</t>
+          <t>O.6</t>
         </is>
       </c>
       <c r="B109" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Max Promo Price Column' to hide it.</t>
+          <t>Click on the preference dropdown icon to open the preference options.</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Max Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr"/>
@@ -2638,17 +2469,17 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>P.11</t>
+          <t>O.7</t>
         </is>
       </c>
       <c r="B110" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the 'Min Promo Price Column' to hide it.</t>
+          <t>Click on 'Save Preference' to save the current column visibility settings.</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("treeitem", name="Min Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr"/>
@@ -2658,17 +2489,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>P.12</t>
+          <t>O.8</t>
         </is>
       </c>
       <c r="B111" s="4" t="inlineStr">
         <is>
-          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible again.</t>
+          <t>Click on the preference dropdown icon again to reopen the preference options.</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
+          <t>`page.locator("div:nth-child(4) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr"/>
@@ -2678,17 +2509,17 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>P.13</t>
+          <t>O.9</t>
         </is>
       </c>
       <c r="B112" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
+          <t>Click on 'Reset Preference' to reset the column visibility settings to their default state.</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
+          <t>`page.get_by_text("Reset Preference").click()`</t>
         </is>
       </c>
       <c r="D112" s="3" t="inlineStr"/>
@@ -2696,39 +2527,26 @@
       <c r="F112" s="4" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>P.14</t>
-        </is>
-      </c>
-      <c r="B113" s="4" t="inlineStr">
-        <is>
-          <t>Fill the 'Filter Columns Input' textbox with the text 'UPC' to filter columns by this keyword.</t>
-        </is>
-      </c>
-      <c r="C113" s="4" t="inlineStr">
-        <is>
-          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("UPC")`</t>
-        </is>
-      </c>
-      <c r="D113" s="3" t="inlineStr"/>
-      <c r="E113" s="4" t="inlineStr"/>
-      <c r="F113" s="4" t="inlineStr"/>
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>--- EXPORT AND PAGINATION INTERACTIONS ---</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>P.15</t>
+          <t>P.1</t>
         </is>
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>Uncheck the visibility toggle for the filtered column matching 'UPC' to hide it.</t>
+          <t>Click on the export icon to initiate the download process.</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
+          <t>`page.locator("div:nth-child(3) &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr"/>
@@ -2738,17 +2556,17 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>P.16</t>
+          <t>P.2</t>
         </is>
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Preference' icon to open the dropdown menu for saving preferences.</t>
+          <t>Click on the first element with the class 'align-middle' to interact with it.</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div:nth-child(2) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
+          <t>`page.locator(".align-middle").first.click()`</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr"/>
@@ -2758,17 +2576,17 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>P.17</t>
+          <t>P.3</t>
         </is>
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>Click on 'Save Preference' to save the current grid settings or preferences.</t>
+          <t>Click on the second occurrence of the text 'Event' to navigate or interact with the Event section.</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("Save Preference").click()`</t>
+          <t>`page.get_by_text("Event").nth(1).click()`</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr"/>
@@ -2778,17 +2596,17 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>P.18</t>
+          <t>P.4</t>
         </is>
       </c>
       <c r="B117" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'Export' icon to initiate the export process and trigger the file download.</t>
+          <t>Click on the button within the 'Event Details columns (0)' card to open column visibility options.</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
+          <t>`page.locator("esp-card-component").filter(has_text="Event Details columns (0)").get_by_role("button").click()`</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr"/>
@@ -2798,17 +2616,17 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>P.19</t>
+          <t>P.5</t>
         </is>
       </c>
       <c r="B118" s="4" t="inlineStr">
         <is>
-          <t>Click on the second page link in the pagination to navigate to the second page of the grid.</t>
+          <t>Uncheck the visibility toggle for the 'Event Column' to hide it.</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("a").nth(2).click()`</t>
+          <t>`page.get_by_role("treeitem", name="Event Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D118" s="3" t="inlineStr"/>
@@ -2818,17 +2636,17 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>P.20</t>
+          <t>P.6</t>
         </is>
       </c>
       <c r="B119" s="4" t="inlineStr">
         <is>
-          <t>Click on the page link labeled '3' to navigate to the third page of the grid.</t>
+          <t>Uncheck the visibility toggle for the 'UPC 12 Column' to hide it.</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("a").filter(has_text="3").click()`</t>
+          <t>`page.get_by_role("treeitem", name="UPC 12 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr"/>
@@ -2838,17 +2656,17 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>P.21</t>
+          <t>P.7</t>
         </is>
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>Click on the 'First Page' button in the pagination controls to navigate back to the first page of the grid.</t>
+          <t>Uncheck the visibility toggle for the 'Customer Level 2 Column' to hide it.</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .card-content &gt; esp-row-dimentional-grid &gt; div &gt; #paginationId &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first").click()`</t>
+          <t>`page.get_by_role("treeitem", name="Customer Level 2 Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr"/>
@@ -2858,17 +2676,17 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>Q.1</t>
+          <t>P.8</t>
         </is>
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>Click on the dropdown labeled 'View 10 row(s)' to open the row display options.</t>
+          <t>Uncheck the visibility toggle for the 'Start Date Column' to hide it.</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_text("View 10 row(s)").nth(2).click()`</t>
+          <t>`page.get_by_role("treeitem", name="Start Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D121" s="3" t="inlineStr"/>
@@ -2878,17 +2696,17 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Q.2</t>
+          <t>P.9</t>
         </is>
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>Select the option 'View 20 row(s)' from the dropdown to change the number of rows displayed.</t>
+          <t>Uncheck the visibility toggle for the 'End Date Column' to hide it.</t>
         </is>
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>`page.locator("div").filter(has_text=re.compile(r"^View 20 row\(s\)$")).nth(1).click()`</t>
+          <t>`page.get_by_role("treeitem", name="End Date Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr"/>
@@ -2898,17 +2716,17 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>Q.3</t>
+          <t>P.10</t>
         </is>
       </c>
       <c r="B123" s="4" t="inlineStr">
         <is>
-          <t>Click on the column header icon to open the filter options for the column.</t>
+          <t>Uncheck the visibility toggle for the 'Max Promo Price Column' to hide it.</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
+          <t>`page.get_by_role("treeitem", name="Max Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D123" s="3" t="inlineStr"/>
@@ -2918,17 +2736,17 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>Q.4</t>
+          <t>P.11</t>
         </is>
       </c>
       <c r="B124" s="4" t="inlineStr">
         <is>
-          <t>Fill the filter textbox with the value 'Promotion' to filter the column based on this value.</t>
+          <t>Uncheck the visibility toggle for the 'Min Promo Price Column' to hide it.</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("textbox", name="Filter Value").fill("Promotion")`</t>
+          <t>`page.get_by_role("treeitem", name="Min Promo Price Column").get_by_label("Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr"/>
@@ -2938,17 +2756,17 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>Q.5</t>
+          <t>P.12</t>
         </is>
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>Click the 'Apply' button to apply the column filter.</t>
+          <t>Check the 'Toggle All Columns Visibility' checkbox to make all columns visible again.</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Toggle All Columns Visibility").check()`</t>
         </is>
       </c>
       <c r="D125" s="3" t="inlineStr"/>
@@ -2958,17 +2776,17 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>Q.6</t>
+          <t>P.13</t>
         </is>
       </c>
       <c r="B126" s="4" t="inlineStr">
         <is>
-          <t>Click on the filtered column header to interact with the column filter settings.</t>
+          <t>Click on the 'Filter Columns Input' textbox to focus on it.</t>
         </is>
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-cell-filtered &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").click()`</t>
         </is>
       </c>
       <c r="D126" s="3" t="inlineStr"/>
@@ -2978,17 +2796,17 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>Q.7</t>
+          <t>P.14</t>
         </is>
       </c>
       <c r="B127" s="4" t="inlineStr">
         <is>
-          <t>Click on the filter icon to open the active filter options for the column.</t>
+          <t>Fill the 'Filter Columns Input' textbox with the text 'UPC' to filter columns by this keyword.</t>
         </is>
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
+          <t>`page.get_by_role("textbox", name="Filter Columns Input").fill("UPC")`</t>
         </is>
       </c>
       <c r="D127" s="3" t="inlineStr"/>
@@ -2998,17 +2816,17 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>Q.8</t>
+          <t>P.15</t>
         </is>
       </c>
       <c r="B128" s="4" t="inlineStr">
         <is>
-          <t>Click the 'Reset' button to clear the applied column filter.</t>
+          <t>Uncheck the visibility toggle for the filtered column matching 'UPC' to hide it.</t>
         </is>
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
+          <t>`page.get_by_role("checkbox", name="Press SPACE to toggle visibility (visible)").uncheck()`</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr"/>
@@ -3018,17 +2836,17 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>R.1</t>
+          <t>P.16</t>
         </is>
       </c>
       <c r="B129" s="4" t="inlineStr">
         <is>
-          <t>Double-click on the grid cell with the name 'Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/' to interact with or edit the cell.</t>
+          <t>Click on the 'Preference' icon to open the dropdown menu for saving preferences.</t>
         </is>
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>`page.get_by_role("gridcell", name="Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/").dblclick()`</t>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div:nth-child(2) &gt; #preference-iconId &gt; .legend-font &gt; .multiselect-dropdown &gt; .pointer").click()`</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr"/>
@@ -3038,17 +2856,17 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>R.2</t>
+          <t>P.17</t>
         </is>
       </c>
       <c r="B130" s="4" t="inlineStr">
         <is>
-          <t>Close the current page after completing the interaction.</t>
+          <t>Click on 'Save Preference' to save the current grid settings or preferences.</t>
         </is>
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>`page.close()`</t>
+          <t>`page.get_by_text("Save Preference").click()`</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr"/>
@@ -3058,17 +2876,17 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>R.3</t>
+          <t>P.18</t>
         </is>
       </c>
       <c r="B131" s="4" t="inlineStr">
         <is>
-          <t>Close the browser context to clean up resources and end the session.</t>
+          <t>Click on the 'Export' icon to initiate the export process and trigger the file download.</t>
         </is>
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>`context.close()`</t>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .title &gt; .grid-icons-container &gt; esp-grid-icons-component &gt; .display-grid-icons &gt; div &gt; #export-iconId &gt; .icon-color-toolbar-active").click()`</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr"/>
@@ -3078,26 +2896,336 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>R.4</t>
+          <t>P.19</t>
         </is>
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>Close the browser instance to terminate all associated contexts and sessions.</t>
+          <t>Click on the second page link in the pagination to navigate to the second page of the grid.</t>
         </is>
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>`browser.close()`</t>
+          <t>`page.locator("a").nth(2).click()`</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr"/>
       <c r="E132" s="4" t="inlineStr"/>
       <c r="F132" s="4" t="inlineStr"/>
     </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>P.20</t>
+        </is>
+      </c>
+      <c r="B133" s="4" t="inlineStr">
+        <is>
+          <t>Click on the page link labeled '3' to navigate to the third page of the grid.</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("a").filter(has_text="3").click()`</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr"/>
+      <c r="E133" s="4" t="inlineStr"/>
+      <c r="F133" s="4" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>P.21</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>Click on the 'First Page' button in the pagination controls to navigate back to the first page of the grid.</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("div:nth-child(7) &gt; div &gt; esp-grid-container &gt; esp-card-component &gt; .card-container &gt; .card-content &gt; esp-row-dimentional-grid &gt; div &gt; #paginationId &gt; esp-pagination-v2 &gt; .d-flex.w-100 &gt; .pagination-pager &gt; .pagination-first").click()`</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr"/>
+      <c r="E134" s="4" t="inlineStr"/>
+      <c r="F134" s="4" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>--- ROW DISPLAY AND COLUMN FILTERING ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Q.1</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>Click on the dropdown labeled 'View 10 row(s)' to open the row display options.</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_text("View 10 row(s)").nth(2).click()`</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr"/>
+      <c r="E136" s="4" t="inlineStr"/>
+      <c r="F136" s="4" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Q.2</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Select the option 'View 20 row(s)' from the dropdown to change the number of rows displayed.</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator("div").filter(has_text=re.compile(r"^View 20 row\(s\)$")).nth(1).click()`</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr"/>
+      <c r="E137" s="4" t="inlineStr"/>
+      <c r="F137" s="4" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>Q.3</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Click on the column header icon to open the filter options for the column.</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-active &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container &gt; .ag-header-icon &gt; .ag-icon").click()`</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr"/>
+      <c r="E138" s="4" t="inlineStr"/>
+      <c r="F138" s="4" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>Q.4</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Fill the filter textbox with the value 'Promotion' to filter the column based on this value.</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("textbox", name="Filter Value").fill("Promotion")`</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr"/>
+      <c r="E139" s="4" t="inlineStr"/>
+      <c r="F139" s="4" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>Q.5</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Click the 'Apply' button to apply the column filter.</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Apply").click()`</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr"/>
+      <c r="E140" s="4" t="inlineStr"/>
+      <c r="F140" s="4" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Click on the filtered column header to interact with the column filter settings.</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".ag-header-cell.ag-header-parent-hidden.ag-header-cell-sortable.ag-header-background.ag-focus-managed.ag-header-cell-filtered &gt; .ag-header-cell-comp-wrapper &gt; .ag-cell-label-container").click()`</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr"/>
+      <c r="E141" s="4" t="inlineStr"/>
+      <c r="F141" s="4" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>Q.7</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>Click on the filter icon to open the active filter options for the column.</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>`page.locator(".ag-header-icon.ag-header-cell-filter-button.ag-filter-active &gt; .ag-icon").click()`</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr"/>
+      <c r="E142" s="4" t="inlineStr"/>
+      <c r="F142" s="4" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>Q.8</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Click the 'Reset' button to clear the applied column filter.</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_label("Column Filter").get_by_role("button", name="Reset").click()`</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr"/>
+      <c r="E143" s="4" t="inlineStr"/>
+      <c r="F143" s="4" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>--- FINAL GRID INTERACTIONS AND CLEANUP ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>R.1</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Double-click on the grid cell with the name 'Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/' to interact with or edit the cell.</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>`page.get_by_role("gridcell", name="Promotion-TH PRO BAGEL ROLLBACK 12/29/25 thru 03/29/").dblclick()`</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr"/>
+      <c r="E145" s="4" t="inlineStr"/>
+      <c r="F145" s="4" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>R.2</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>Close the current page after completing the interaction.</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>`page.close()`</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr"/>
+      <c r="E146" s="4" t="inlineStr"/>
+      <c r="F146" s="4" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>R.3</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Close the browser context to clean up resources and end the session.</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>`context.close()`</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr"/>
+      <c r="E147" s="4" t="inlineStr"/>
+      <c r="F147" s="4" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>R.4</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Close the browser instance to terminate all associated contexts and sessions.</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>`browser.close()`</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr"/>
+      <c r="E148" s="4" t="inlineStr"/>
+      <c r="F148" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="17">
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A92:F92"/>
+    <mergeCell ref="A113:F113"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A103:F103"/>
+    <mergeCell ref="A144:F144"/>
+    <mergeCell ref="A135:F135"/>
+    <mergeCell ref="A83:F83"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>